<commit_message>
auto: sync reports 2026-05-05 15:58
</commit_message>
<xml_diff>
--- a/feedback-reports/Full-Stack_Development_with_GenAI_Honours_Program.xlsx
+++ b/feedback-reports/Full-Stack_Development_with_GenAI_Honours_Program.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nandita.vora\OneDrive - NIIT Limited\NIIT-AI Powered FSE - General\Design Docs\FSE-v6\Feedback-App\feedback-reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="300" documentId="11_71F05A531246E64FEE670415535DCE3AA7C4B014" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BD311E8-C13C-4CAA-813A-050E3DB618DE}"/>
+  <xr:revisionPtr revIDLastSave="302" documentId="11_71F05A531246E64FEE670415535DCE3AA7C4B014" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{E88C2044-D968-4508-A85F-A5DA46ADCF1B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,23 +23,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="184">
   <si>
     <t>Program Name</t>
   </si>
@@ -1089,6 +1078,12 @@
   </si>
   <si>
     <t>Remarks</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>suggestion fixed</t>
   </si>
 </sst>
 </file>
@@ -2538,7 +2533,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="49" spans="1:7">
+    <row r="49" spans="1:8">
       <c r="A49" s="3">
         <v>46</v>
       </c>
@@ -2556,7 +2551,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="79.2">
+    <row r="50" spans="1:8" ht="79.2">
       <c r="A50" s="3">
         <v>47</v>
       </c>
@@ -2574,7 +2569,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="26.4">
+    <row r="51" spans="1:8" ht="26.4">
       <c r="A51" s="3">
         <v>48</v>
       </c>
@@ -2594,7 +2589,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="52" spans="1:7">
+    <row r="52" spans="1:8">
       <c r="A52" s="3">
         <v>49</v>
       </c>
@@ -2612,7 +2607,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="53" spans="1:7">
+    <row r="53" spans="1:8">
       <c r="A53" s="3">
         <v>50</v>
       </c>
@@ -2630,7 +2625,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="138">
+    <row r="54" spans="1:8" ht="138">
       <c r="A54" s="3">
         <v>51</v>
       </c>
@@ -2648,7 +2643,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:8">
       <c r="A55" s="3">
         <v>52</v>
       </c>
@@ -2666,7 +2661,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="92.4">
+    <row r="56" spans="1:8" ht="92.4">
       <c r="A56" s="3">
         <v>53</v>
       </c>
@@ -2684,7 +2679,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="66">
+    <row r="57" spans="1:8" ht="66">
       <c r="A57" s="3">
         <v>54</v>
       </c>
@@ -2704,7 +2699,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="58" spans="1:7" ht="52.8">
+    <row r="58" spans="1:8" ht="52.8">
       <c r="A58" s="3">
         <v>55</v>
       </c>
@@ -2722,7 +2717,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="39.6">
+    <row r="59" spans="1:8" ht="39.6">
       <c r="A59" s="3">
         <v>56</v>
       </c>
@@ -2741,8 +2736,14 @@
       <c r="F59" s="3" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" ht="39.6">
+      <c r="G59" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="39.6">
       <c r="A60" s="3">
         <v>57</v>
       </c>
@@ -2760,7 +2761,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="61" spans="1:7" ht="171.6">
+    <row r="61" spans="1:8" ht="171.6">
       <c r="A61" s="3">
         <v>58</v>
       </c>
@@ -2781,7 +2782,7 @@
       </c>
       <c r="G61" s="6"/>
     </row>
-    <row r="62" spans="1:7" ht="52.8">
+    <row r="62" spans="1:8" ht="52.8">
       <c r="A62" s="3">
         <v>59</v>
       </c>
@@ -2972,18 +2973,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3005,25 +3006,25 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B34EA2C4-2285-4497-A663-7BC8A09FEAFD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B384905-33E6-4B60-BC29-CDB45CE8B04B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="8b8ad293-1655-4b1e-95cd-578b981aff66"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B384905-33E6-4B60-BC29-CDB45CE8B04B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B34EA2C4-2285-4497-A663-7BC8A09FEAFD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="8b8ad293-1655-4b1e-95cd-578b981aff66"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>